<commit_message>
docs(test): cập nhật bộ test case → 62 TC (thêm 9 commit base vừa sync)
Bổ sung sau merge sync-base: dấu tàu ẢNH GHIM TÀU CÁ (TC_007 sửa + TC_049-051) ·
cảnh báo ranh giới theo vùng VMS admin đổi được + đo mép ngoài + fix báo oan
cảng VN + cờ applies trong-bờ-thì-im (TC_052-057) · nhãn quãng/hướng đường kẻ
tàu→con trỏ (TC_058-059) · nhắc cài PWA song song CH Play (TC_060-062).

48 → 62 TC. Functional 35 · UI 9 · Resilience 9 · Security 4 · Compatibility 3 ·
Validation 2. Phủ toàn bộ chức năng mới + fix của session + 9 commit base.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SDFish_TC_cac-chuc-nang-moi_2026-08-27.xlsx
+++ b/docs/test-cases/SDFish_TC_cac-chuc-nang-moi_2026-08-27.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="353">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -162,18 +162,18 @@
     <t>TC_007</t>
   </si>
   <si>
-    <t>Phân biệt được vị trí tàu (icon tàu) và con trỏ (ghim)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bước 1: Bật GPS/có vị trí → hiện chấm tàu
+    <t>Phân biệt vị trí tàu (ảnh ghim tàu cá) và con trỏ (ghim)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Bật GPS/có vị trí → hiện dấu tàu
 Bước 2: Chạm nơi khác để đặt con trỏ
-Bước 3: So 2 biểu tượng</t>
-  </si>
-  <si>
-    <t>Đã có vị trí GPS (chấm tàu hiện)</t>
-  </si>
-  <si>
-    <t>Vị trí tàu = biểu tượng ICON TÀU; con trỏ = CÁI GHIM; hai hình khác nhau rõ, có đường kẻ nối tàu → con trỏ</t>
+Bước 3: So 2 biểu tượng + đường kẻ nối</t>
+  </si>
+  <si>
+    <t>Đã có vị trí GPS (dấu tàu hiện)</t>
+  </si>
+  <si>
+    <t>Vị trí tàu = ẢNH GHIM TÀU CÁ; con trỏ = CÁI GHIM (khác hình/màu); có đường kẻ nối tàu → con trỏ kèm nhãn quãng + hướng</t>
   </si>
   <si>
     <t>TC_008</t>
@@ -897,6 +897,254 @@
   </si>
   <si>
     <t>Ảnh vẫn hiện đầy đủ sau khi mở lại app (đọc từ Storage qua đường dẫn đã lưu)</t>
+  </si>
+  <si>
+    <t>TC_049</t>
+  </si>
+  <si>
+    <t>SDFish - Ra khơi - Dấu tàu (ảnh ghim tàu cá)</t>
+  </si>
+  <si>
+    <t>Dấu tàu hiện ẢNH GHIM TÀU CÁ, mũi ghim rơi đúng toạ độ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Vào Ra khơi, có vị trí GPS
+Bước 2: Quan sát dấu vị trí tàu trên bản đồ</t>
+  </si>
+  <si>
+    <t>Đã có vị trí GPS</t>
+  </si>
+  <si>
+    <t>Dấu tàu là ẢNH GHIM TÀU CÁ (mũi ghim chỉ xuống); MŨI ghim rơi đúng toạ độ; có quầng nhấp nháy neo vào mũi ghim</t>
+  </si>
+  <si>
+    <t>TC_050</t>
+  </si>
+  <si>
+    <t>Dấu tàu (ghim) KHÔNG xoay theo hướng chạy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Đang chạy tàu / đổi hướng di chuyển
+Bước 2: Quan sát dấu tàu</t>
+  </si>
+  <si>
+    <t>Đang có vị trí + di chuyển</t>
+  </si>
+  <si>
+    <t>Ảnh ghim tàu GIỮ NGUYÊN chiều (mũi chỉ xuống), KHÔNG xoay/nghiêng theo hướng chạy (ghim xoay là nằm nghiêng, mũi rời chỗ)</t>
+  </si>
+  <si>
+    <t>TC_051</t>
+  </si>
+  <si>
+    <t>Mất sóng vẫn thấy dấu tàu (ảnh trong CRITICAL_SHELL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Mở app khi có sóng 1 lần (để cache)
+Bước 2: Ra biển mất sóng, mở Ra khơi</t>
+  </si>
+  <si>
+    <t>Ảnh ghim đã được cache (đã mở app lúc có sóng)</t>
+  </si>
+  <si>
+    <t>Mất sóng vẫn hiện được ảnh ghim tàu (ảnh nằm trong CRITICAL_SHELL của service worker), không mất dấu tàu giữa biển</t>
+  </si>
+  <si>
+    <t>TC_052</t>
+  </si>
+  <si>
+    <t>SDFish - Ra khơi - Cảnh báo ranh giới theo vùng VMS (admin + độ chính xác)</t>
+  </si>
+  <si>
+    <t>Admin đánh dấu vùng VMS là 'ranh giới cảnh báo' (is_border)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Vào /quan-tri → tab Vùng biển
+Bước 2: Trên 1 vùng, bấm nút 'Là ranh giới cảnh báo' (hoặc tick trong form thêm vùng)
+Bước 3: Lưu</t>
+  </si>
+  <si>
+    <t>Đăng nhập ADMIN; migration 0052 (vms_zones.is_border) đã apply prod</t>
+  </si>
+  <si>
+    <t>1 vùng VMS dạng vùng KÍN (polygon)</t>
+  </si>
+  <si>
+    <t>Vùng được đánh dấu is_border=true; app ngư dân dùng HÌNH vùng này làm ranh giới cảnh báo (thay dữ liệu tĩnh)</t>
+  </si>
+  <si>
+    <t>Vùng đó định nghĩa ranh giới cảnh báo</t>
+  </si>
+  <si>
+    <t>TC_053</t>
+  </si>
+  <si>
+    <t>Không đánh dấu vùng nào → app dùng ranh giới tĩnh (hành vi không đổi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Đảm bảo KHÔNG vùng VMS nào bật is_border
+Bước 2: Vào Ra khơi, xem cảnh báo ranh giới</t>
+  </si>
+  <si>
+    <t>Không vùng nào is_border=true (hoặc cột chưa apply)</t>
+  </si>
+  <si>
+    <t>App dùng ranh giới TĨNH (src/data) như cũ — hành vi cảnh báo không đổi (đường lùi an toàn, không phải lỗi)</t>
+  </si>
+  <si>
+    <t>TC_054</t>
+  </si>
+  <si>
+    <t>Cảng cá VN KHÔNG bị báo oan 'đã ngoài ranh giới'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Đưa/giả lập vị trí tàu tại một cảng cá VN (vd Vũng Tàu, Thọ Quang)
+Bước 2: Xem cảnh báo ranh giới</t>
+  </si>
+  <si>
+    <t>Ở Ra khơi</t>
+  </si>
+  <si>
+    <t>Toạ độ cảng cá VN trong bờ</t>
+  </si>
+  <si>
+    <t>KHÔNG hiện câu 'đã ngoài ranh giới'; điểm trong bờ/trong vùng cho phép được coi là hợp lệ (đã sửa lỗi báo oan trước đây)</t>
+  </si>
+  <si>
+    <t>TC_055</t>
+  </si>
+  <si>
+    <t>Điểm trong bờ thì IM — không in khoảng cách tới biên</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Trỏ tới / ở một điểm nằm trong bờ (không ra biển)
+Bước 2: Xem thông tin khoảng cách tới biên</t>
+  </si>
+  <si>
+    <t>Điểm trong bờ</t>
+  </si>
+  <si>
+    <t>KHÔNG in khoảng cách tới biên cho điểm trong bờ (cờ applies=false) — tránh con số vô nghĩa</t>
+  </si>
+  <si>
+    <t>TC_056</t>
+  </si>
+  <si>
+    <t>Ra ngoài mép vùng VMS → báo 'đã ngoài biên'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Có vùng VMS kín được đánh dấu is_border
+Bước 2: Đưa vị trí tàu RA NGOÀI mép vùng đó (phía biển)
+Bước 3: Xem cảnh báo</t>
+  </si>
+  <si>
+    <t>Có vùng kín is_border=true; đang Dẫn đường</t>
+  </si>
+  <si>
+    <t>Vị trí ngoài mép vùng VMS</t>
+  </si>
+  <si>
+    <t>Đo khoảng cách tới MÉP NGOÀI vùng; khi ra ngoài (phía biển) hiện 'đã ngoài ranh giới' — chỉ khi có vùng KÍN mới dám khẳng định trong/ngoài</t>
+  </si>
+  <si>
+    <t>TC_057</t>
+  </si>
+  <si>
+    <t>Nguồn chỉ có ĐƯỜNG (không vùng kín) → không khẳng định trong/ngoài</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Chỉ có đường biên (LineString), không có vùng kín is_border
+Bước 2: Xem cảnh báo khi gần biên</t>
+  </si>
+  <si>
+    <t>Nguồn ranh giới chỉ là đường</t>
+  </si>
+  <si>
+    <t>Vẫn đo được KHOẢNG CÁCH tới biên, nhưng KHÔNG hiện câu 'đã ngoài ranh giới' (đường hở không có 'bên trong')</t>
+  </si>
+  <si>
+    <t>TC_058</t>
+  </si>
+  <si>
+    <t>SDFish - Ra khơi - Nhãn quãng + hướng trên đường kẻ tàu → con trỏ</t>
+  </si>
+  <si>
+    <t>Đường kẻ tàu → con trỏ có nhãn quãng + hướng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Có vị trí tàu (GPS)
+Bước 2: Chạm 1 điểm để trỏ tới
+Bước 3: Xem đường kẻ nối tàu → con trỏ</t>
+  </si>
+  <si>
+    <t>Đường kẻ tàu → con trỏ hiện NHÃN gồm quãng (hải lý) + hướng (độ/hướng VN) ngay trên đường</t>
+  </si>
+  <si>
+    <t>TC_059</t>
+  </si>
+  <si>
+    <t>Không có vị trí tàu → không vẽ đường kẻ (không lấy cảng/tâm màn thay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Chưa có vị trí GPS (chưa cấp quyền / mất định vị)
+Bước 2: Trỏ tới 1 điểm</t>
+  </si>
+  <si>
+    <t>Chưa có vị trí tàu</t>
+  </si>
+  <si>
+    <t>KHÔNG vẽ đường kẻ tàu → con trỏ (không biết tàu ở đâu thì không có đầu để kẻ); không lấy cảng nhà/tâm màn hình thay thế</t>
+  </si>
+  <si>
+    <t>TC_060</t>
+  </si>
+  <si>
+    <t>SDFish - Chung - Nhắc cài app (PWA) song song CH Play</t>
+  </si>
+  <si>
+    <t>Nhắc cài PWA hiện được kể cả khi có bản CH Play</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Mở app trên trình duyệt (chưa cài PWA)
+Bước 2: Quan sát băng nhắc 'Cài về máy'</t>
+  </si>
+  <si>
+    <t>Chưa cài PWA; đang dùng qua trình duyệt</t>
+  </si>
+  <si>
+    <t>Băng nhắc 'Cài về máy' hiện được (không còn phụ thuộc sự kiện beforeinstallprompt); Android hướng dẫn cài kể cả khi đã có bản trên CH Play</t>
+  </si>
+  <si>
+    <t>TC_061</t>
+  </si>
+  <si>
+    <t>Đã cài (standalone) → ẩn nhắc cài</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Mở app đã cài về màn hình chính (chế độ standalone)
+Bước 2: Quan sát</t>
+  </si>
+  <si>
+    <t>App đã cài (standalone)</t>
+  </si>
+  <si>
+    <t>KHÔNG hiện băng nhắc cài (đã cài rồi thì thôi)</t>
+  </si>
+  <si>
+    <t>TC_062</t>
+  </si>
+  <si>
+    <t>Bấm tắt / cài-rồi-huỷ → ngừng nhắc, không nhắc quá số lần</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bước 1: Bấm X trên băng nhắc cài (hoặc chọn cài rồi huỷ)
+Bước 2: Mở lại app nhiều lần</t>
+  </si>
+  <si>
+    <t>Đang hiện băng nhắc cài</t>
+  </si>
+  <si>
+    <t>Sau khi tắt → ngừng nhắc; không nhắc lại quá số lần/khoảng cách đã định (không làm phiền)</t>
   </si>
 </sst>
 </file>
@@ -1317,7 +1565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -3115,9 +3363,521 @@
         <v>19</v>
       </c>
     </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L50" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B51" s="3"/>
+      <c r="C51" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L51" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B52" s="3"/>
+      <c r="C52" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="L52" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="I53" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L53" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B54" s="3"/>
+      <c r="C54" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I54" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="L54" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B55" s="3"/>
+      <c r="C55" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I55" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L55" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="B56" s="3"/>
+      <c r="C56" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L56" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="B57" s="3"/>
+      <c r="C57" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L57" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B58" s="3"/>
+      <c r="C58" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="H58" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I58" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L58" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="H59" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I59" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L59" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B60" s="3"/>
+      <c r="C60" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G60" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="H60" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I60" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L60" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="H61" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I61" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L61" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="B62" s="3"/>
+      <c r="C62" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="H62" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I62" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="L62" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B63" s="3"/>
+      <c r="C63" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G63" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="H63" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I63" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L63" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L49"/>
-  <mergeCells count="8">
+  <autoFilter ref="A1:L63"/>
+  <mergeCells count="12">
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B9:B13"/>
@@ -3126,6 +3886,10 @@
     <mergeCell ref="B27:B35"/>
     <mergeCell ref="B36:B39"/>
     <mergeCell ref="B40:B49"/>
+    <mergeCell ref="B50:B52"/>
+    <mergeCell ref="B53:B58"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="B61:B63"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>